<commit_message>
ajoute role agent de saisie
</commit_message>
<xml_diff>
--- a/public/docs/exemplaires-import-biens/exemplaire_blocs_immeubles.xlsx
+++ b/public/docs/exemplaires-import-biens/exemplaire_blocs_immeubles.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AD2211-197D-4D06-A2AA-1F8ED5A6D875}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D4EE5C-DC36-42DA-99FF-4D8A189007EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Bloc</t>
   </si>
@@ -119,13 +119,49 @@
   </si>
   <si>
     <t>Superficie vendable</t>
+  </si>
+  <si>
+    <t>GH01</t>
+  </si>
+  <si>
+    <t>GH02</t>
+  </si>
+  <si>
+    <t>GH03</t>
+  </si>
+  <si>
+    <t>IMM01</t>
+  </si>
+  <si>
+    <t>IMM02</t>
+  </si>
+  <si>
+    <t>IMM03</t>
+  </si>
+  <si>
+    <t>RDC</t>
+  </si>
+  <si>
+    <t>1er étage</t>
+  </si>
+  <si>
+    <t>2ème étage</t>
+  </si>
+  <si>
+    <t>B01</t>
+  </si>
+  <si>
+    <t>B02</t>
+  </si>
+  <si>
+    <t>B03</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,6 +173,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -451,12 +493,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AG4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="8.90625" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="7" width="22.90625" customWidth="1"/>
@@ -582,7 +624,50 @@
         <v>31</v>
       </c>
     </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>